<commit_message>
Part changed in LCSC Electrode Board BOM S.No 1
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Electrode-Board/LCSC_BOM_Electrode_Board.xlsx
+++ b/Deliverables/BOM/Electrode-Board/LCSC_BOM_Electrode_Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\ManarHarake-sEMGDevice\Deliverables\BOM\Electrode-Board\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9934645-EE68-4C68-8C19-44BF0646E6EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78804275-6DB2-4BEE-A6A3-CEC4F4C3328A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,9 +44,6 @@
     <t>C307331</t>
   </si>
   <si>
-    <t>C2922482</t>
-  </si>
-  <si>
     <t>C325464</t>
   </si>
   <si>
@@ -72,6 +69,9 @@
   </si>
   <si>
     <t>C110221</t>
+  </si>
+  <si>
+    <t>C91606</t>
   </si>
 </sst>
 </file>
@@ -606,7 +606,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C2" s="5">
         <v>50</v>
@@ -628,7 +628,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C4" s="5">
         <v>100</v>
@@ -639,7 +639,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C5" s="12">
         <v>50</v>
@@ -650,7 +650,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C6" s="5">
         <v>100</v>
@@ -661,7 +661,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C7" s="9">
         <v>100</v>
@@ -672,7 +672,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C8" s="5">
         <v>300</v>
@@ -683,7 +683,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C9" s="9">
         <v>100</v>
@@ -694,7 +694,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C10" s="5">
         <v>45</v>
@@ -705,7 +705,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C11" s="9">
         <v>100</v>
@@ -716,7 +716,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12" s="11">
         <v>42</v>

</xml_diff>